<commit_message>
V9: make v9 regenerado (etiquetas de D1 corregidas en cifras_clave)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDwCFFTud391ebBMaJpdsw
</commit_message>
<xml_diff>
--- a/output/v9/tablas_v9.xlsx
+++ b/output/v9/tablas_v9.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>zonas tensionadas (Ley 12/2023): ATT sobre contratos de contratos nuevos (CS)</t>
+          <t>zonas tensionadas (Ley 12/2023): diferencia (ATT, CS) en el número de contratos nuevos</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -741,7 +741,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>zonas tensionadas (Ley 12/2023): ATT sobre renta media de contratos nuevos (CS)</t>
+          <t>zonas tensionadas (Ley 12/2023): diferencia (ATT, CS) en la renta media de los contratos nuevos</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -980,7 +980,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ley catalana 11/2020: ATT sobre contratos de contratos nuevos (CS)</t>
+          <t>Ley catalana 11/2020: diferencia (ATT, CS) en el número de contratos nuevos</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Ley catalana 11/2020: ATT sobre renta media de contratos nuevos (CS)</t>
+          <t>Ley catalana 11/2020: diferencia (ATT, CS) en la renta media de los contratos nuevos</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">

</xml_diff>